<commit_message>
fix(settle): reconcile Spark + Grove per-venue positions vs BA Labs (Jan→May 2026) (#112)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -652,7 +652,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-05T00:25:53+00:00</t>
+          <t>2026-06-05T11:08:01+00:00</t>
         </is>
       </c>
     </row>
@@ -1354,10 +1354,10 @@
         </is>
       </c>
       <c r="E10" s="5" t="n">
-        <v>0</v>
+        <v>49900000</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>0</v>
+        <v>49900000</v>
       </c>
       <c r="G10" s="5" t="n">
         <v>0</v>

</xml_diff>

<commit_message>
feat(grove): address Grove findings — Maple syrupUSDC, Agora incentives, daily Debt xlsx tab (#117)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -11,8 +11,9 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-protocol holdings" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE daily" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-protocol holdings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE daily" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -76,7 +77,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="10">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -89,6 +90,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -652,7 +654,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-05T11:08:01+00:00</t>
+          <t>2026-06-08T08:17:40+00:00</t>
         </is>
       </c>
     </row>
@@ -679,7 +681,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S30"/>
+  <dimension ref="A1:S32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -2058,12 +2060,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E37</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Curve AUSD/USDC stableswap LP</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2073,7 +2075,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
@@ -2123,12 +2125,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle)</t>
+          <t>Curve AUSD/USDC stableswap LP</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2138,7 +2140,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -2188,12 +2190,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E16</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>DAI raw (ALM idle)</t>
+          <t>RLUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -2253,12 +2255,12 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>E17</t>
+          <t>E16</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
+          <t>DAI raw (ALM idle)</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
@@ -2296,7 +2298,7 @@
         <v>0</v>
       </c>
       <c r="M24" s="6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="N24" s="5" t="n">
         <v>0</v>
@@ -2313,21 +2315,17 @@
       <c r="R24" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S24" t="inlineStr">
-        <is>
-          <t>CoF excluded (already deducted from utilized)</t>
-        </is>
-      </c>
+      <c r="S24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>E18</t>
+          <t>E17</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
+          <t>USDS raw / POL (ALM idle — already netted out of utilized)</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -2337,7 +2335,7 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E25" s="5" t="n">
@@ -2365,7 +2363,7 @@
         <v>0</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" s="5" t="n">
         <v>0</v>
@@ -2382,22 +2380,26 @@
       <c r="R25" s="5" t="n">
         <v>0</v>
       </c>
-      <c r="S25" t="inlineStr"/>
+      <c r="S25" t="inlineStr">
+        <is>
+          <t>CoF excluded (already deducted from utilized)</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>E23</t>
+          <t>E18</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Steakhouse Prime Instant (Base, Morpho V2)</t>
+          <t>sUSDS raw / POL (ALM idle — Cat B 4626)</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
@@ -2452,17 +2454,17 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>E24</t>
+          <t>E23</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
+          <t>Steakhouse Prime Instant (Base, Morpho V2)</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>ethereum</t>
+          <t>base</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2517,12 +2519,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>E26</t>
+          <t>E24</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>PYUSD raw (ALM idle)</t>
+          <t>Steakhouse High Yield PYUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -2532,7 +2534,7 @@
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E28" s="5" t="n">
@@ -2582,17 +2584,17 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>E27</t>
+          <t>E26</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>USDC raw on Base (ALM idle)</t>
+          <t>PYUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>base</t>
+          <t>ethereum</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
@@ -2647,59 +2649,189 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
+          <t>E27</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>USDC raw on Base (ALM idle)</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>base</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S30" t="inlineStr"/>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>E38</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>Agora AUSD incentives (cash distribution to Grove Eth ALM)</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>ethereum</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="N31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S31" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
           <t>PSM_CURVE_DEDUCT</t>
         </is>
       </c>
-      <c r="B30" t="inlineStr">
+      <c r="B32" t="inlineStr">
         <is>
           <t>PSM3 USDS + PSM3 USDC (SDE) + Curve idle USDS — BR deduction (unattributed)</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="F30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="G30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="H30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="I30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="J30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="K30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="L30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="M30" s="6" t="n">
-        <v>0</v>
-      </c>
-      <c r="N30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="O30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="P30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="Q30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="R30" s="5" t="n">
-        <v>0</v>
-      </c>
-      <c r="S30" t="inlineStr">
+      <c r="C32" t="inlineStr"/>
+      <c r="D32" t="inlineStr"/>
+      <c r="E32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="J32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="K32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>0</v>
+      </c>
+      <c r="N32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="O32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="P32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="R32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="S32" t="inlineStr">
         <is>
           <t>BR deduction from PSM3 USDS leg + PSM3 USDC leg (SDE, ≈$0 yield) + Curve idle USDS — not tracked per-venue; residual = sky_rev_br_reduction − Σ(known venue deduction_avg × effective_br_rate × n_days)</t>
         </is>
@@ -3145,6 +3277,1671 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:O38"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="16" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="10" max="10"/>
+    <col width="11" customWidth="1" min="11" max="11"/>
+    <col width="12" customWidth="1" min="12" max="12"/>
+    <col width="11" customWidth="1" min="13" max="13"/>
+    <col width="18" customWidth="1" min="14" max="14"/>
+    <col width="22" customWidth="1" min="15" max="15"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Daily ilk debt + Sky charge breakdown</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="45" customHeight="1">
+      <c r="A3" s="9" t="inlineStr">
+        <is>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="2" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B5" s="2" t="inlineStr">
+        <is>
+          <t>cum_debt</t>
+        </is>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>− ALM idle</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>− PSM USDS</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="inlineStr">
+        <is>
+          <t>− SDE NAV</t>
+        </is>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>− Curve idle</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr">
+        <is>
+          <t>− Lending idle</t>
+        </is>
+      </c>
+      <c r="H5" s="2">
+        <f> utilized</f>
+        <v/>
+      </c>
+      <c r="I5" s="2" t="inlineStr">
+        <is>
+          <t>SSR APY</t>
+        </is>
+      </c>
+      <c r="J5" s="2" t="inlineStr">
+        <is>
+          <t>base APY</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr">
+        <is>
+          <t>T (months)</t>
+        </is>
+      </c>
+      <c r="L5" s="2" t="inlineStr">
+        <is>
+          <t>ref_rate APY</t>
+        </is>
+      </c>
+      <c r="M5" s="2" t="inlineStr">
+        <is>
+          <t>sub APY</t>
+        </is>
+      </c>
+      <c r="N5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge</t>
+        </is>
+      </c>
+      <c r="O5" s="2" t="inlineStr">
+        <is>
+          <t>daily Sky charge (gross on cum_debt)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>1984828055.219324</v>
+      </c>
+      <c r="C6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="5" t="n">
+        <v>762824824.7566538</v>
+      </c>
+      <c r="F6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>1222003230.46267</v>
+      </c>
+      <c r="I6" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J6" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M6" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N6" s="3" t="n">
+        <v>124430.2757766502</v>
+      </c>
+      <c r="O6" s="3" t="n">
+        <v>212664.3707622077</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>2026-01-02</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>762860738.2166537</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>1222967317.00267</v>
+      </c>
+      <c r="I7" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J7" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M7" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N7" s="3" t="n">
+        <v>124541.7893254808</v>
+      </c>
+      <c r="O7" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>2026-01-03</t>
+        </is>
+      </c>
+      <c r="B8" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="5" t="n">
+        <v>762860738.2166537</v>
+      </c>
+      <c r="F8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>1222967317.00267</v>
+      </c>
+      <c r="I8" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J8" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M8" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N8" s="3" t="n">
+        <v>124541.7893254808</v>
+      </c>
+      <c r="O8" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>2026-01-04</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="n">
+        <v>1985828055.219324</v>
+      </c>
+      <c r="C9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="5" t="n">
+        <v>762900103.7688839</v>
+      </c>
+      <c r="F9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>1222927951.45044</v>
+      </c>
+      <c r="I9" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J9" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M9" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N9" s="3" t="n">
+        <v>124537.2360076522</v>
+      </c>
+      <c r="O9" s="3" t="n">
+        <v>212780.0383337419</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>2026-01-05</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="n">
+        <v>1995828055.219324</v>
+      </c>
+      <c r="C10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="5" t="n">
+        <v>763022687.8884877</v>
+      </c>
+      <c r="F10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H10" s="5" t="n">
+        <v>1232805367.330836</v>
+      </c>
+      <c r="I10" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J10" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M10" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N10" s="3" t="n">
+        <v>125679.7327155704</v>
+      </c>
+      <c r="O10" s="3" t="n">
+        <v>213936.7140490833</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>2026-01-06</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="n">
+        <v>2012328055.219324</v>
+      </c>
+      <c r="C11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="5" t="n">
+        <v>763063046.3086326</v>
+      </c>
+      <c r="F11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H11" s="5" t="n">
+        <v>1249265008.910691</v>
+      </c>
+      <c r="I11" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J11" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M11" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N11" s="3" t="n">
+        <v>127583.5794854346</v>
+      </c>
+      <c r="O11" s="3" t="n">
+        <v>215845.2289793966</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>2026-01-07</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>2006577041.234456</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>803105106.0675159</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H12" s="5" t="n">
+        <v>1203471935.16694</v>
+      </c>
+      <c r="I12" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J12" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M12" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N12" s="3" t="n">
+        <v>122286.8058524111</v>
+      </c>
+      <c r="O12" s="3" t="n">
+        <v>215180.023157908</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>2026-01-08</t>
+        </is>
+      </c>
+      <c r="B13" s="5" t="n">
+        <v>2026577041.234456</v>
+      </c>
+      <c r="C13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="5" t="n">
+        <v>803143978.3027297</v>
+      </c>
+      <c r="F13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>1223433062.931726</v>
+      </c>
+      <c r="I13" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J13" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M13" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N13" s="3" t="n">
+        <v>124595.6610260466</v>
+      </c>
+      <c r="O13" s="3" t="n">
+        <v>217493.3745885908</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>2026-01-09</t>
+        </is>
+      </c>
+      <c r="B14" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I14" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J14" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M14" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N14" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O14" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>2026-01-10</t>
+        </is>
+      </c>
+      <c r="B15" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I15" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J15" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M15" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N15" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O15" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>2026-01-11</t>
+        </is>
+      </c>
+      <c r="B16" s="5" t="n">
+        <v>1926524960.710924</v>
+      </c>
+      <c r="C16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="5" t="n">
+        <v>823185735.0412451</v>
+      </c>
+      <c r="F16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G16" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>1103339225.669679</v>
+      </c>
+      <c r="I16" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J16" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K16" t="n">
+        <v>0</v>
+      </c>
+      <c r="L16" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M16" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N16" s="3" t="n">
+        <v>110704.6985137294</v>
+      </c>
+      <c r="O16" s="3" t="n">
+        <v>205920.5934074957</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>2026-01-12</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="n">
+        <v>1956524960.710924</v>
+      </c>
+      <c r="C17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="5" t="n">
+        <v>843317637.3667084</v>
+      </c>
+      <c r="F17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>1113207323.344216</v>
+      </c>
+      <c r="I17" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J17" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K17" t="n">
+        <v>0</v>
+      </c>
+      <c r="L17" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M17" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N17" s="3" t="n">
+        <v>111846.1174074048</v>
+      </c>
+      <c r="O17" s="3" t="n">
+        <v>209390.6205535199</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-01-13</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="n">
+        <v>1946290696.105259</v>
+      </c>
+      <c r="C18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="5" t="n">
+        <v>903358721.0850873</v>
+      </c>
+      <c r="F18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>1042931975.020172</v>
+      </c>
+      <c r="I18" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J18" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K18" t="n">
+        <v>0</v>
+      </c>
+      <c r="L18" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M18" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N18" s="3" t="n">
+        <v>103717.5385280469</v>
+      </c>
+      <c r="O18" s="3" t="n">
+        <v>208206.8480201448</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>2026-01-14</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="n">
+        <v>1971790696.105259</v>
+      </c>
+      <c r="C19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="5" t="n">
+        <v>903399116.9614611</v>
+      </c>
+      <c r="F19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>1068391579.143798</v>
+      </c>
+      <c r="I19" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J19" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K19" t="n">
+        <v>0</v>
+      </c>
+      <c r="L19" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M19" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N19" s="3" t="n">
+        <v>106662.3891092473</v>
+      </c>
+      <c r="O19" s="3" t="n">
+        <v>211156.3710942654</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>2026-01-15</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="5" t="n">
+        <v>943446845.432757</v>
+      </c>
+      <c r="F20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>1018329389.021003</v>
+      </c>
+      <c r="I20" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J20" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K20" t="n">
+        <v>0</v>
+      </c>
+      <c r="L20" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M20" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N20" s="3" t="n">
+        <v>100871.8171520632</v>
+      </c>
+      <c r="O20" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>2026-01-16</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G21" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I21" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J21" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K21" t="n">
+        <v>0</v>
+      </c>
+      <c r="L21" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M21" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N21" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O21" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>2026-01-17</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G22" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I22" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J22" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K22" t="n">
+        <v>0</v>
+      </c>
+      <c r="L22" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M22" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N22" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O22" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>2026-01-18</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="n">
+        <v>1961776234.45376</v>
+      </c>
+      <c r="C23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>1018275743.78463</v>
+      </c>
+      <c r="I23" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J23" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K23" t="n">
+        <v>0</v>
+      </c>
+      <c r="L23" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M23" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N23" s="3" t="n">
+        <v>100865.6121378476</v>
+      </c>
+      <c r="O23" s="3" t="n">
+        <v>209998.0226348147</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>2026-01-19</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="n">
+        <v>1962777234.45376</v>
+      </c>
+      <c r="C24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="5" t="n">
+        <v>943500490.6691302</v>
+      </c>
+      <c r="F24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H24" s="5" t="n">
+        <v>1019276743.78463</v>
+      </c>
+      <c r="I24" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J24" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K24" t="n">
+        <v>0</v>
+      </c>
+      <c r="L24" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M24" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N24" s="3" t="n">
+        <v>100981.3953769532</v>
+      </c>
+      <c r="O24" s="3" t="n">
+        <v>210113.8058739204</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>2026-01-20</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="n">
+        <v>1933909642.799006</v>
+      </c>
+      <c r="C25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="5" t="n">
+        <v>963737271.2934443</v>
+      </c>
+      <c r="F25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H25" s="5" t="n">
+        <v>970172371.5055617</v>
+      </c>
+      <c r="I25" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J25" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K25" t="n">
+        <v>0</v>
+      </c>
+      <c r="L25" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M25" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N25" s="3" t="n">
+        <v>95806.17217862917</v>
+      </c>
+      <c r="O25" s="3" t="n">
+        <v>206774.7616511758</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>2026-01-21</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="n">
+        <v>1934309642.799006</v>
+      </c>
+      <c r="C26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="5" t="n">
+        <v>983792436.63439</v>
+      </c>
+      <c r="F26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H26" s="5" t="n">
+        <v>950517206.164616</v>
+      </c>
+      <c r="I26" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J26" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K26" t="n">
+        <v>0</v>
+      </c>
+      <c r="L26" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M26" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N26" s="3" t="n">
+        <v>93865.19116313005</v>
+      </c>
+      <c r="O26" s="3" t="n">
+        <v>206821.0286797895</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>2026-01-22</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="n">
+        <v>1972909642.799006</v>
+      </c>
+      <c r="C27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="5" t="n">
+        <v>983848621.2736028</v>
+      </c>
+      <c r="F27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>989061021.5254031</v>
+      </c>
+      <c r="I27" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J27" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K27" t="n">
+        <v>0</v>
+      </c>
+      <c r="L27" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M27" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N27" s="3" t="n">
+        <v>97671.45850214559</v>
+      </c>
+      <c r="O27" s="3" t="n">
+        <v>211285.7969410072</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>2026-01-23</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="n">
+        <v>1972909642.799006</v>
+      </c>
+      <c r="C28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" s="5" t="n">
+        <v>983907696.0662968</v>
+      </c>
+      <c r="F28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G28" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H28" s="5" t="n">
+        <v>989001946.7327092</v>
+      </c>
+      <c r="I28" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J28" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K28" t="n">
+        <v>0</v>
+      </c>
+      <c r="L28" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M28" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N28" s="3" t="n">
+        <v>97665.62476586687</v>
+      </c>
+      <c r="O28" s="3" t="n">
+        <v>211285.7969410072</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>2026-01-24</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="n">
+        <v>1974009642.799006</v>
+      </c>
+      <c r="C29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" s="5" t="n">
+        <v>1003909435.032003</v>
+      </c>
+      <c r="F29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G29" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H29" s="5" t="n">
+        <v>970100207.7670031</v>
+      </c>
+      <c r="I29" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J29" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K29" t="n">
+        <v>0</v>
+      </c>
+      <c r="L29" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M29" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N29" s="3" t="n">
+        <v>95799.04588667894</v>
+      </c>
+      <c r="O29" s="3" t="n">
+        <v>211413.0312696948</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>2026-01-25</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="n">
+        <v>1974009642.799006</v>
+      </c>
+      <c r="C30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" s="5" t="n">
+        <v>1003909435.032003</v>
+      </c>
+      <c r="F30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G30" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H30" s="5" t="n">
+        <v>970100207.7670031</v>
+      </c>
+      <c r="I30" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J30" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K30" t="n">
+        <v>0</v>
+      </c>
+      <c r="L30" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M30" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N30" s="3" t="n">
+        <v>95799.04588667894</v>
+      </c>
+      <c r="O30" s="3" t="n">
+        <v>211413.0312696948</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>2026-01-26</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="n">
+        <v>2007509642.799006</v>
+      </c>
+      <c r="C31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" s="5" t="n">
+        <v>1004098132.792144</v>
+      </c>
+      <c r="F31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G31" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>1003411510.006862</v>
+      </c>
+      <c r="I31" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J31" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K31" t="n">
+        <v>0</v>
+      </c>
+      <c r="L31" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M31" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N31" s="3" t="n">
+        <v>99146.30231405739</v>
+      </c>
+      <c r="O31" s="3" t="n">
+        <v>215287.8949160884</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>2026-01-27</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="n">
+        <v>2007509642.799006</v>
+      </c>
+      <c r="C32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E32" s="5" t="n">
+        <v>1024159461.833279</v>
+      </c>
+      <c r="F32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G32" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H32" s="5" t="n">
+        <v>983350180.9657269</v>
+      </c>
+      <c r="I32" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J32" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K32" t="n">
+        <v>0</v>
+      </c>
+      <c r="L32" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M32" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N32" s="3" t="n">
+        <v>97107.50328138829</v>
+      </c>
+      <c r="O32" s="3" t="n">
+        <v>215287.8949160884</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>2026-01-28</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="n">
+        <v>2027509642.799006</v>
+      </c>
+      <c r="C33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" s="5" t="n">
+        <v>1024225089.412934</v>
+      </c>
+      <c r="F33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G33" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H33" s="5" t="n">
+        <v>1003284553.386072</v>
+      </c>
+      <c r="I33" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J33" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K33" t="n">
+        <v>0</v>
+      </c>
+      <c r="L33" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M33" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N33" s="3" t="n">
+        <v>99131.61755004049</v>
+      </c>
+      <c r="O33" s="3" t="n">
+        <v>217601.2463467712</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>2026-01-29</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" s="5" t="n">
+        <v>1044281848.307186</v>
+      </c>
+      <c r="F34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G34" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H34" s="5" t="n">
+        <v>1005279794.49182</v>
+      </c>
+      <c r="I34" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J34" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K34" t="n">
+        <v>0</v>
+      </c>
+      <c r="L34" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M34" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N34" s="3" t="n">
+        <v>99362.40224336745</v>
+      </c>
+      <c r="O34" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>2026-01-30</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" s="5" t="n">
+        <v>1064349366.450599</v>
+      </c>
+      <c r="F35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G35" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>985212276.3484071</v>
+      </c>
+      <c r="I35" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J35" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K35" t="n">
+        <v>0</v>
+      </c>
+      <c r="L35" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M35" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N35" s="3" t="n">
+        <v>97291.38836829222</v>
+      </c>
+      <c r="O35" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>2026-01-31</t>
+        </is>
+      </c>
+      <c r="B36" s="5" t="n">
+        <v>2049561642.799006</v>
+      </c>
+      <c r="C36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" s="5" t="n">
+        <v>1064349366.450599</v>
+      </c>
+      <c r="F36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="G36" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="H36" s="5" t="n">
+        <v>985212276.3484071</v>
+      </c>
+      <c r="I36" s="6" t="n">
+        <v>0.04</v>
+      </c>
+      <c r="J36" s="6" t="n">
+        <v>0.04312</v>
+      </c>
+      <c r="K36" t="n">
+        <v>0</v>
+      </c>
+      <c r="L36" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="M36" s="6" t="n">
+        <v>0.0367</v>
+      </c>
+      <c r="N36" s="3" t="n">
+        <v>97291.38836829222</v>
+      </c>
+      <c r="O36" s="3" t="n">
+        <v>220151.9476342421</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="8" t="inlineStr">
+        <is>
+          <t>Σ daily charges</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr"/>
+      <c r="C38" t="inlineStr"/>
+      <c r="D38" t="inlineStr"/>
+      <c r="E38" t="inlineStr"/>
+      <c r="F38" t="inlineStr"/>
+      <c r="G38" t="inlineStr"/>
+      <c r="H38" t="inlineStr"/>
+      <c r="I38" t="inlineStr"/>
+      <c r="J38" t="inlineStr"/>
+      <c r="K38" t="inlineStr"/>
+      <c r="L38" t="inlineStr"/>
+      <c r="M38" t="inlineStr"/>
+      <c r="N38" s="10" t="n">
+        <v>3322924.199551741</v>
+      </c>
+      <c r="O38" s="10" t="n">
+        <v>6577707.668676052</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:I13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -3438,7 +5235,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>

<commit_message>
settlements(grove): re-render Jan–May 2026 xlsx after rebase
Numbers byte-identical to main (Grove uses ALLOCATOR-BLOOM-A with
``rate ≡ 1``, so the daily Vat-rate scaling is a no-op for this prime):
prime_agent_total_revenue=$22,182,542.35, sky_revenue=$36,646,535.24
cumulative Jan–May 2026.

Only the xlsx display changed: the Debt tab note now describes
``cum_debt`` as rate-scaled (mathematically a no-op here but consistent
with the methodology after the SPARK-A fix), and the Sky Revenue tab
sUSDS spread label is corrected to "deducted from sky_revenue".

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -654,7 +654,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-08T08:17:40+00:00</t>
+          <t>2026-06-09T00:20:43+00:00</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40), then scaled by Vat.ilks[ilk].rate_d / 1e27 read at each day's EoD block — actual outstanding USDS per day, not raw normalised Art. utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Fix/debt timeseries calculation (#121)
Co-authored-by: Cursor <cursoragent@cursor.com>
Co-authored-by: lakonema2000 <lakonema2000@gmail.com>
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -654,7 +654,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-08T08:17:40+00:00</t>
+          <t>2026-06-09T00:20:43+00:00</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40). utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40), then scaled by Vat.ilks[ilk].rate_d / 1e27 read at each day's EoD block — actual outstanding USDS per day, not raw normalised Art. utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
fix(spark+grove): Spark agent_rate $0 (wrong subproxy address) + Grove E23 $3.27M phantom revenue (Dune indexing gap) (#124)
Co-authored-by: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -489,7 +489,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3270233.03914781</v>
+        <v>3270233.046142676</v>
       </c>
     </row>
     <row r="5">
@@ -505,7 +505,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3276508.564995402</v>
+        <v>3276508.571990268</v>
       </c>
     </row>
     <row r="8">
@@ -603,7 +603,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>3270233.03914781</v>
+        <v>3270233.046142676</v>
       </c>
     </row>
     <row r="20">
@@ -619,7 +619,7 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>-52691.16040393031</v>
+        <v>-52691.15340906432</v>
       </c>
     </row>
     <row r="23">
@@ -654,7 +654,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-09T00:20:43+00:00</t>
+          <t>2026-06-09T16:55:07+00:00</t>
         </is>
       </c>
     </row>
@@ -851,13 +851,13 @@
         <v>0.3949353765426448</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>667436.8242189552</v>
+        <v>667436.8242190982</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2097307.007608659</v>
+        <v>2097307.007608802</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>265862.3596886521</v>
+        <v>265862.3596885091</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>325000000</v>
@@ -989,13 +989,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>804560.318340226</v>
+        <v>804560.3183403984</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>804560.318340226</v>
+        <v>804560.3183403984</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>240035.7880645352</v>
+        <v>240035.7880643629</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1054,13 +1054,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>782299.7924869618</v>
+        <v>782299.7924871293</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>782299.7924869618</v>
+        <v>782299.7924871293</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-547300.2259265231</v>
+        <v>-547300.2259266907</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1188,13 +1188,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>315433.0125244209</v>
+        <v>315433.0125244884</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>315433.0125244209</v>
+        <v>315433.0125244884</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>300954.8874755791</v>
+        <v>300954.8874755116</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1253,13 +1253,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>230521.3983884985</v>
+        <v>230521.3983885479</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>230521.3983884985</v>
+        <v>230521.3983885479</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-124801.5258788677</v>
+        <v>-124801.5258789171</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1318,13 +1318,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>160722.5734720856</v>
+        <v>160722.57347212</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>160722.5734720856</v>
+        <v>160722.57347212</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>-91502.87925664459</v>
+        <v>-91502.87925667902</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1383,13 +1383,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>157716.5062622104</v>
+        <v>157716.5062622442</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>157716.5062622104</v>
+        <v>157716.5062622442</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>51419.74373778956</v>
+        <v>51419.74373775578</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1452,13 +1452,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78858.25313110522</v>
+        <v>78858.25313112211</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78858.25313110522</v>
+        <v>78858.25313112211</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-78858.25313110522</v>
+        <v>-78858.25313112211</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1521,13 +1521,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>78148.0817562388</v>
+        <v>78148.08175625555</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>78148.0817562388</v>
+        <v>78148.08175625555</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-76760.90542223879</v>
+        <v>-76760.90542225554</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1586,13 +1586,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>35689.80639782174</v>
+        <v>35689.80639782939</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>35689.80639782174</v>
+        <v>35689.80639782939</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>8322.663590178259</v>
+        <v>8322.663590170614</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1633,31 +1633,31 @@
         <v>1009793.258152034</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>10040.61065874401</v>
+        <v>10040.61765361</v>
       </c>
       <c r="I14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J14" s="5" t="n">
-        <v>10040.61065874401</v>
+        <v>10040.61765361</v>
       </c>
       <c r="K14" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L14" s="5" t="n">
-        <v>3225721.217461766</v>
+        <v>3225721.217236125</v>
       </c>
       <c r="M14" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10174.98961187907</v>
+        <v>10174.98961116951</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>10174.98961187907</v>
+        <v>10174.98961116951</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-134.3789531350658</v>
+        <v>-134.371957559508</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1716,13 +1716,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1322.807708632826</v>
+        <v>1322.80770863311</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1322.807708632826</v>
+        <v>1322.80770863311</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>17.9909305529012</v>
+        <v>17.99093055261786</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1781,13 +1781,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>21.38301216424558</v>
+        <v>21.38301216425016</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>21.38301216424558</v>
+        <v>21.38301216425016</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-21.38301216274558</v>
+        <v>-21.38301216275016</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1846,13 +1846,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>18.45199404192008</v>
+        <v>18.45199404192403</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>18.45199404192008</v>
+        <v>18.45199404192403</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-3613.91545804192</v>
+        <v>-3613.915458041924</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1911,10 +1911,10 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.0002464982819673339</v>
+        <v>0.0002464982819673867</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.0002464982819673339</v>
+        <v>0.0002464982819673867</v>
       </c>
       <c r="P18" s="5" t="n">
         <v>3688.873147501718</v>

</xml_diff>

<commit_message>
fix(rates): de-freeze SSR + refresh EFFR, surface subsidy benefit (Spark Jan–May: Sky −$2.3M / Spark +$2.3M) (#137)
Co-authored-by: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -22,10 +22,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="3">
+  <numFmts count="4">
     <numFmt numFmtId="164" formatCode="&quot;$&quot;#,##0.00;&quot;−$&quot;#,##0.00;&quot;$&quot;0.00"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0;&quot;−$&quot;#,##0;&quot;$&quot;0"/>
     <numFmt numFmtId="166" formatCode="0.000%"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
   </numFmts>
   <fonts count="4">
     <font>
@@ -77,7 +78,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -85,12 +86,14 @@
     <xf numFmtId="164" fontId="2" fillId="0" borderId="1" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="166" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="166" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="164" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -499,13 +502,13 @@
         </is>
       </c>
       <c r="B5" s="3" t="n">
-        <v>6275.525847591615</v>
+        <v>6275.526124407053</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3276508.571990268</v>
+        <v>3276508.572267083</v>
       </c>
     </row>
     <row r="8">
@@ -527,7 +530,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3322924.199551741</v>
+        <v>3322924.21170079</v>
       </c>
     </row>
     <row r="10">
@@ -543,7 +546,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>6277336.076888746</v>
+        <v>6277336.089037795</v>
       </c>
     </row>
     <row r="13">
@@ -565,7 +568,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>3322924.199551741</v>
+        <v>3322924.21170079</v>
       </c>
     </row>
     <row r="15">
@@ -575,13 +578,13 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-3254783.469124312</v>
+        <v>-3254783.608419782</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" s="4" t="n">
-        <v>6577707.668676052</v>
+        <v>6577707.820120571</v>
       </c>
     </row>
     <row r="18">
@@ -613,13 +616,13 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>-3322924.199551741</v>
+        <v>-3322924.21170079</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>-52691.15340906432</v>
+        <v>-52691.16555811382</v>
       </c>
     </row>
     <row r="23">
@@ -654,7 +657,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-06-10T15:01:19+00:00</t>
+          <t>2026-06-23T21:34:35+00:00</t>
         </is>
       </c>
     </row>
@@ -851,13 +854,13 @@
         <v>0.3949353765426448</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>667436.8242190982</v>
+        <v>667436.8266593353</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2097307.007608802</v>
+        <v>2097307.010049039</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>265862.3596885091</v>
+        <v>265862.357248272</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>325000000</v>
@@ -989,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>804560.3183403984</v>
+        <v>804560.3212819771</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>804560.3183403984</v>
+        <v>804560.3212819771</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>240035.7880643629</v>
+        <v>240035.7851227842</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1054,13 +1057,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>782299.7924871293</v>
+        <v>782299.7953473206</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>782299.7924871293</v>
+        <v>782299.7953473206</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-547300.2259266907</v>
+        <v>-547300.228786882</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1188,13 +1191,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>315433.0125244884</v>
+        <v>315433.0136777532</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>315433.0125244884</v>
+        <v>315433.0136777532</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>300954.8874755116</v>
+        <v>300954.8863222468</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1253,13 +1256,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>230521.3983885479</v>
+        <v>230521.3992313645</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>230521.3983885479</v>
+        <v>230521.3992313645</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-124801.5258789171</v>
+        <v>-124801.5267217337</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1318,13 +1321,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>160722.57347212</v>
+        <v>160722.5740597429</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>160722.57347212</v>
+        <v>160722.5740597429</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>-91502.87925667902</v>
+        <v>-91502.87984430196</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1383,13 +1386,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>157716.5062622442</v>
+        <v>157716.5068388766</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>157716.5062622442</v>
+        <v>157716.5068388766</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>51419.74373775578</v>
+        <v>51419.74316112341</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1452,13 +1455,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78858.25313112211</v>
+        <v>78858.25341943829</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78858.25313112211</v>
+        <v>78858.25341943829</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-78858.25313112211</v>
+        <v>-78858.25341943829</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1521,13 +1524,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>78148.08175625555</v>
+        <v>78148.08204197524</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>78148.08175625555</v>
+        <v>78148.08204197524</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-76760.90542225554</v>
+        <v>-76760.90570797524</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1586,13 +1589,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>35689.80639782939</v>
+        <v>35689.80652831603</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>35689.80639782939</v>
+        <v>35689.80652831603</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>8322.663590170614</v>
+        <v>8322.66345968397</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1651,13 +1654,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10174.98961116951</v>
+        <v>10174.98964837061</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>10174.98961116951</v>
+        <v>10174.98964837061</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-134.371957559508</v>
+        <v>-134.3719947606131</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1716,13 +1719,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1322.80770863311</v>
+        <v>1322.807713469469</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1322.80770863311</v>
+        <v>1322.807713469469</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>17.99093055261786</v>
+        <v>17.99092571625827</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1781,13 +1784,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>21.38301216425016</v>
+        <v>21.38301224242928</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>21.38301216425016</v>
+        <v>21.38301224242928</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-21.38301216275016</v>
+        <v>-21.38301224092928</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1846,13 +1849,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>18.45199404192403</v>
+        <v>18.45199410938696</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>18.45199404192403</v>
+        <v>18.45199410938696</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-3613.915458041924</v>
+        <v>-3613.915458109387</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1911,13 +1914,13 @@
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.0002464982819673867</v>
+        <v>0.000246498282868617</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.0002464982819673867</v>
+        <v>0.000246498282868617</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>3688.873147501718</v>
+        <v>3688.873147501717</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -2848,7 +2851,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B24"/>
+  <dimension ref="A1:C44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="80" customWidth="1" min="1" max="1"/>
@@ -2863,185 +2866,367 @@
       </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="inlineStr">
-        <is>
-          <t>Component</t>
-        </is>
-      </c>
-      <c r="B3" s="2" t="inlineStr">
-        <is>
-          <t>USD</t>
+      <c r="A3" s="7" t="inlineStr">
+        <is>
+          <t>Rates &amp; subsidy — effective rate charged this period</t>
         </is>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>CoF on utilized debt (= Σ_d max(utilized_d,0) × (1+BR_d)^(1/365)−1)</t>
-        </is>
-      </c>
-      <c r="B4" s="3" t="n">
-        <v>3322924.199551741</v>
+      <c r="A4" s="2" t="inlineStr">
+        <is>
+          <t>Metric</t>
+        </is>
+      </c>
+      <c r="B4" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>+ Sky-Direct revenue (full venue yield on fixed/capped SDE)</t>
-        </is>
-      </c>
-      <c r="B5" s="3" t="n">
-        <v>2954411.877337005</v>
+          <t>Time-weighted utilized</t>
+        </is>
+      </c>
+      <c r="B5" s="5" t="n">
+        <v>1071984731.030483</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>equals sky_revenue (total Sky take this month)</t>
-        </is>
-      </c>
-      <c r="B6" s="3" t="n">
-        <v>6277336.076888746</v>
+          <t xml:space="preserve">  — first $1B (subsidised tranche)</t>
+        </is>
+      </c>
+      <c r="B6" s="5" t="n">
+        <v>993313796.6169302</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  — excess (full base-rate tranche)</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>78670934.41355301</v>
       </c>
     </row>
     <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>Utilized base = cum_debt − idle USDS − PSM USDS − Σ SDE asset value − Curve idle − lending idle</t>
-        </is>
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>Base rate (BR = SSR + 30bps), period avg</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="n">
+        <v>0.04312000189646037</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="inlineStr">
+        <is>
+          <t>Reference rate (tbill_3m), period avg</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="n">
+        <v>0.0367</v>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="8" t="inlineStr">
-        <is>
-          <t>Sky Revenue (max) — BR × full ilk debt (no deductions)</t>
-        </is>
-      </c>
-      <c r="B10" s="3" t="n">
-        <v>6577707.668676052</v>
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>Subsidised rate (BR*), period avg</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="n">
+        <v>0.0367</v>
       </c>
     </row>
     <row r="11">
-      <c r="A11" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ↳ actual CoF on Net_Subs (BR × utilized)</t>
-        </is>
-      </c>
-      <c r="B11" s="3" t="n">
-        <v>3322924.199551741</v>
+      <c r="A11" s="7" t="inlineStr">
+        <is>
+          <t>Effective blended rate charged</t>
+        </is>
+      </c>
+      <c r="B11" s="8" t="n">
+        <v>0.03717115181169214</v>
       </c>
     </row>
     <row r="12">
-      <c r="A12" t="inlineStr">
-        <is>
-          <t xml:space="preserve">    ↳ reduction from idle/SDE deductions</t>
-        </is>
-      </c>
-      <c r="B12" s="3" t="n">
-        <v>-3254783.469124312</v>
-      </c>
-    </row>
-    <row r="13" ht="60" customHeight="1">
-      <c r="A13" s="9" t="inlineStr">
-        <is>
-          <t>Note: sky_revenue can EXCEED sky_revenue_gross for primes with active SDE positions — sky_revenue also adds sde_revenue on top of BR-on-utilized. The subsidised BR (ref_rate ramp) is already applied here; this is NOT the raw Maker base rate.</t>
-        </is>
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Diff vs base rate (bps)</t>
+        </is>
+      </c>
+      <c r="B12" s="9" t="n">
+        <v>-59.48850084768234</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="7" t="inlineStr">
+        <is>
+          <t>Subsidy benefit to prime (USD)</t>
+        </is>
+      </c>
+      <c r="B13" s="10" t="n">
+        <v>520885.9412035887</v>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Subsidy</t>
-        </is>
-      </c>
-      <c r="B15" s="2" t="inlineStr">
-        <is>
-          <t>Value</t>
-        </is>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>CoF at full base rate (no subsidy)</t>
+        </is>
+      </c>
+      <c r="B15" s="3" t="n">
+        <v>3843810.152904379</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>enabled</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>true</t>
-        </is>
+          <t xml:space="preserve">  − actual CoF (subsidy on first tranche)</t>
+        </is>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>3322924.21170079</v>
       </c>
     </row>
     <row r="17">
-      <c r="A17" t="inlineStr">
-        <is>
-          <t>cap_usd</t>
-        </is>
-      </c>
-      <c r="B17" s="5" t="n">
-        <v>1000000000</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="inlineStr">
-        <is>
-          <t>program_start</t>
-        </is>
-      </c>
-      <c r="B18" t="inlineStr">
-        <is>
-          <t>2026-01-01</t>
-        </is>
+      <c r="A17" s="7" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  = subsidy benefit</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="n">
+        <v>520885.9412035887</v>
       </c>
     </row>
     <row r="19">
-      <c r="A19" t="inlineStr">
-        <is>
-          <t>ramp_months</t>
-        </is>
-      </c>
-      <c r="B19" t="n">
-        <v>24</v>
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Tranche</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr">
+        <is>
+          <t>Avg balance</t>
+        </is>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>CoF (USD)</t>
+        </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>ref_rate_kind</t>
-        </is>
-      </c>
-      <c r="B20" t="inlineStr">
-        <is>
-          <t>tbill_3m</t>
-        </is>
+          <t>Subsidised (first $1B)</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="n">
+        <v>993313796.6169302</v>
+      </c>
+      <c r="C20" s="3" t="n">
+        <v>3040834.245599687</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
+          <t>Excess (&gt; cap)</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="n">
+        <v>78670934.41355301</v>
+      </c>
+      <c r="C21" s="3" t="n">
+        <v>282089.9661011035</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t>Component</t>
+        </is>
+      </c>
+      <c r="B23" s="2" t="inlineStr">
+        <is>
+          <t>USD</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>CoF on utilized debt (= Σ_d max(utilized_d,0) × (1+BR_d)^(1/365)−1)</t>
+        </is>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>3322924.21170079</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>+ Sky-Direct revenue (full venue yield on fixed/capped SDE)</t>
+        </is>
+      </c>
+      <c r="B25" s="3" t="n">
+        <v>2954411.877337005</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>equals sky_revenue (total Sky take this month)</t>
+        </is>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>6277336.089037795</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="11" t="inlineStr">
+        <is>
+          <t>Utilized base = cum_debt − idle USDS − PSM USDS − Σ SDE asset value − Curve idle − lending idle</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="7" t="inlineStr">
+        <is>
+          <t>Sky Revenue (max) — BR × full ilk debt (no deductions)</t>
+        </is>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>6577707.820120571</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ↳ actual CoF on Net_Subs (BR × utilized)</t>
+        </is>
+      </c>
+      <c r="B31" s="3" t="n">
+        <v>3322924.21170079</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t xml:space="preserve">    ↳ reduction from idle/SDE deductions</t>
+        </is>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>-3254783.608419782</v>
+      </c>
+    </row>
+    <row r="33" ht="60" customHeight="1">
+      <c r="A33" s="12" t="inlineStr">
+        <is>
+          <t>Note: sky_revenue can EXCEED sky_revenue_gross for primes with active SDE positions — sky_revenue also adds sde_revenue on top of BR-on-utilized. The subsidised BR (ref_rate ramp) is already applied here; this is NOT the raw Maker base rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="2" t="inlineStr">
+        <is>
+          <t>Subsidy</t>
+        </is>
+      </c>
+      <c r="B35" s="2" t="inlineStr">
+        <is>
+          <t>Value</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>enabled</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>true</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>cap_usd</t>
+        </is>
+      </c>
+      <c r="B37" s="5" t="n">
+        <v>1000000000</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>program_start</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>2026-01-01</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>ramp_months</t>
+        </is>
+      </c>
+      <c r="B39" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>ref_rate_kind</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>tbill_3m</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
           <t>T this period</t>
         </is>
       </c>
-      <c r="B21" t="inlineStr">
+      <c r="B41" t="inlineStr">
         <is>
           <t>0 (SoM) → 0 (EoM)</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="7" t="inlineStr">
+    <row r="42">
+      <c r="A42" s="11" t="inlineStr">
         <is>
           <t>Formula</t>
         </is>
       </c>
-      <c r="B22" t="inlineStr">
+      <c r="B42" t="inlineStr">
         <is>
           <t>subsidised_apy = ref_rate + (base_apy − ref_rate) × min(T, 24) / 24, applied to first cap_usd of utilized; excess at full base_apy</t>
         </is>
       </c>
     </row>
-    <row r="24">
-      <c r="A24" s="7" t="inlineStr">
+    <row r="44">
+      <c r="A44" s="11" t="inlineStr">
         <is>
           <t>Base rate composition: base_apy = (1 + SSR)(1 + 30bps) − 1 (multiplicative)</t>
         </is>
@@ -3305,7 +3490,7 @@
       </c>
     </row>
     <row r="3" ht="45" customHeight="1">
-      <c r="A3" s="9" t="inlineStr">
+      <c r="A3" s="12" t="inlineStr">
         <is>
           <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40), then scaled by Vat.ilks[ilk].rate_d / 1e27 read at each day's EoD block — actual outstanding USDS per day, not raw normalised Art. utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
@@ -3415,10 +3600,10 @@
         <v>1222003230.46267</v>
       </c>
       <c r="I6" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J6" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K6" t="n">
         <v>0</v>
@@ -3430,10 +3615,10 @@
         <v>0.0367</v>
       </c>
       <c r="N6" s="3" t="n">
-        <v>124430.2757766502</v>
+        <v>124430.276882575</v>
       </c>
       <c r="O6" s="3" t="n">
-        <v>212664.3707622077</v>
+        <v>212664.3756681983</v>
       </c>
     </row>
     <row r="7">
@@ -3464,10 +3649,10 @@
         <v>1222967317.00267</v>
       </c>
       <c r="I7" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J7" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K7" t="n">
         <v>0</v>
@@ -3479,10 +3664,10 @@
         <v>0.0367</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>124541.7893254808</v>
+        <v>124541.7904362082</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>212780.0383337419</v>
+        <v>212780.043244714</v>
       </c>
     </row>
     <row r="8">
@@ -3513,10 +3698,10 @@
         <v>1222967317.00267</v>
       </c>
       <c r="I8" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J8" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K8" t="n">
         <v>0</v>
@@ -3528,10 +3713,10 @@
         <v>0.0367</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>124541.7893254808</v>
+        <v>124541.7904362082</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>212780.0383337419</v>
+        <v>212780.043244714</v>
       </c>
     </row>
     <row r="9">
@@ -3562,10 +3747,10 @@
         <v>1222927951.45044</v>
       </c>
       <c r="I9" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J9" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K9" t="n">
         <v>0</v>
@@ -3577,10 +3762,10 @@
         <v>0.0367</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>124537.2360076522</v>
+        <v>124537.2371181835</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>212780.0383337419</v>
+        <v>212780.043244714</v>
       </c>
     </row>
     <row r="10">
@@ -3611,10 +3796,10 @@
         <v>1232805367.330836</v>
       </c>
       <c r="I10" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J10" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K10" t="n">
         <v>0</v>
@@ -3626,10 +3811,10 @@
         <v>0.0367</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>125679.7327155704</v>
+        <v>125679.7338753068</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>213936.7140490833</v>
+        <v>213936.7190098711</v>
       </c>
     </row>
     <row r="11">
@@ -3660,10 +3845,10 @@
         <v>1249265008.910691</v>
       </c>
       <c r="I11" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J11" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K11" t="n">
         <v>0</v>
@@ -3675,10 +3860,10 @@
         <v>0.0367</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>127583.5794854346</v>
+        <v>127583.5807271658</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>215845.2289793966</v>
+        <v>215845.2340223803</v>
       </c>
     </row>
     <row r="12">
@@ -3709,10 +3894,10 @@
         <v>1203471935.16694</v>
       </c>
       <c r="I12" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J12" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K12" t="n">
         <v>0</v>
@@ -3724,10 +3909,10 @@
         <v>0.0367</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>122286.8058524111</v>
+        <v>122286.8068660209</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>215180.023157908</v>
+        <v>215180.0281722427</v>
       </c>
     </row>
     <row r="13">
@@ -3758,10 +3943,10 @@
         <v>1223433062.931726</v>
       </c>
       <c r="I13" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J13" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K13" t="n">
         <v>0</v>
@@ -3773,10 +3958,10 @@
         <v>0.0367</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>124595.6610260466</v>
+        <v>124595.6621390942</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>217493.3745885908</v>
+        <v>217493.3797025569</v>
       </c>
     </row>
     <row r="14">
@@ -3807,10 +3992,10 @@
         <v>1103339225.669679</v>
       </c>
       <c r="I14" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J14" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K14" t="n">
         <v>0</v>
@@ -3822,10 +4007,10 @@
         <v>0.0367</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>110704.6985137294</v>
+        <v>110704.6990285211</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>205920.5934074957</v>
+        <v>205920.5980230453</v>
       </c>
     </row>
     <row r="15">
@@ -3856,10 +4041,10 @@
         <v>1103339225.669679</v>
       </c>
       <c r="I15" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J15" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K15" t="n">
         <v>0</v>
@@ -3871,10 +4056,10 @@
         <v>0.0367</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>110704.6985137294</v>
+        <v>110704.6990285211</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>205920.5934074957</v>
+        <v>205920.5980230453</v>
       </c>
     </row>
     <row r="16">
@@ -3905,10 +4090,10 @@
         <v>1103339225.669679</v>
       </c>
       <c r="I16" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J16" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K16" t="n">
         <v>0</v>
@@ -3920,10 +4105,10 @@
         <v>0.0367</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>110704.6985137294</v>
+        <v>110704.6990285211</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>205920.5934074957</v>
+        <v>205920.5980230453</v>
       </c>
     </row>
     <row r="17">
@@ -3954,10 +4139,10 @@
         <v>1113207323.344216</v>
       </c>
       <c r="I17" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J17" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K17" t="n">
         <v>0</v>
@@ -3969,10 +4154,10 @@
         <v>0.0367</v>
       </c>
       <c r="N17" s="3" t="n">
-        <v>111846.1174074048</v>
+        <v>111846.1179713551</v>
       </c>
       <c r="O17" s="3" t="n">
-        <v>209390.6205535199</v>
+        <v>209390.6253185166</v>
       </c>
     </row>
     <row r="18">
@@ -4003,10 +4188,10 @@
         <v>1042931975.020172</v>
       </c>
       <c r="I18" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J18" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K18" t="n">
         <v>0</v>
@@ -4018,10 +4203,10 @@
         <v>0.0367</v>
       </c>
       <c r="N18" s="3" t="n">
-        <v>103717.5385280469</v>
+        <v>103717.5387419155</v>
       </c>
       <c r="O18" s="3" t="n">
-        <v>208206.8480201448</v>
+        <v>208206.8527341588</v>
       </c>
     </row>
     <row r="19">
@@ -4052,10 +4237,10 @@
         <v>1068391579.143798</v>
       </c>
       <c r="I19" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J19" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K19" t="n">
         <v>0</v>
@@ -4067,10 +4252,10 @@
         <v>0.0367</v>
       </c>
       <c r="N19" s="3" t="n">
-        <v>106662.3891092473</v>
+        <v>106662.3894499448</v>
       </c>
       <c r="O19" s="3" t="n">
-        <v>211156.3710942654</v>
+        <v>211156.3759353094</v>
       </c>
     </row>
     <row r="20">
@@ -4101,10 +4286,10 @@
         <v>1018329389.021003</v>
       </c>
       <c r="I20" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J20" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K20" t="n">
         <v>0</v>
@@ -4116,10 +4301,10 @@
         <v>0.0367</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>100871.8171520632</v>
+        <v>100871.8172433724</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>209998.0226348147</v>
+        <v>209998.027425971</v>
       </c>
     </row>
     <row r="21">
@@ -4150,10 +4335,10 @@
         <v>1018275743.78463</v>
       </c>
       <c r="I21" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J21" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K21" t="n">
         <v>0</v>
@@ -4165,10 +4350,10 @@
         <v>0.0367</v>
       </c>
       <c r="N21" s="3" t="n">
-        <v>100865.6121378476</v>
+        <v>100865.6122288895</v>
       </c>
       <c r="O21" s="3" t="n">
-        <v>209998.0226348147</v>
+        <v>209998.027425971</v>
       </c>
     </row>
     <row r="22">
@@ -4199,10 +4384,10 @@
         <v>1018275743.78463</v>
       </c>
       <c r="I22" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J22" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K22" t="n">
         <v>0</v>
@@ -4214,10 +4399,10 @@
         <v>0.0367</v>
       </c>
       <c r="N22" s="3" t="n">
-        <v>100865.6121378476</v>
+        <v>100865.6122288895</v>
       </c>
       <c r="O22" s="3" t="n">
-        <v>209998.0226348147</v>
+        <v>209998.027425971</v>
       </c>
     </row>
     <row r="23">
@@ -4248,10 +4433,10 @@
         <v>1018275743.78463</v>
       </c>
       <c r="I23" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J23" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K23" t="n">
         <v>0</v>
@@ -4263,10 +4448,10 @@
         <v>0.0367</v>
       </c>
       <c r="N23" s="3" t="n">
-        <v>100865.6121378476</v>
+        <v>100865.6122288895</v>
       </c>
       <c r="O23" s="3" t="n">
-        <v>209998.0226348147</v>
+        <v>209998.027425971</v>
       </c>
     </row>
     <row r="24">
@@ -4297,10 +4482,10 @@
         <v>1019276743.78463</v>
       </c>
       <c r="I24" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J24" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K24" t="n">
         <v>0</v>
@@ -4312,10 +4497,10 @@
         <v>0.0367</v>
       </c>
       <c r="N24" s="3" t="n">
-        <v>100981.3953769532</v>
+        <v>100981.3954729817</v>
       </c>
       <c r="O24" s="3" t="n">
-        <v>210113.8058739204</v>
+        <v>210113.8106700632</v>
       </c>
     </row>
     <row r="25">
@@ -4346,10 +4531,10 @@
         <v>970172371.5055617</v>
       </c>
       <c r="I25" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J25" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K25" t="n">
         <v>0</v>
@@ -4364,7 +4549,7 @@
         <v>95806.17217862917</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>206774.7616511758</v>
+        <v>206774.7663035127</v>
       </c>
     </row>
     <row r="26">
@@ -4395,10 +4580,10 @@
         <v>950517206.164616</v>
       </c>
       <c r="I26" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J26" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K26" t="n">
         <v>0</v>
@@ -4413,7 +4598,7 @@
         <v>93865.19116313005</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>206821.0286797895</v>
+        <v>206821.033334119</v>
       </c>
     </row>
     <row r="27">
@@ -4444,10 +4629,10 @@
         <v>989061021.5254031</v>
       </c>
       <c r="I27" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J27" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K27" t="n">
         <v>0</v>
@@ -4462,7 +4647,7 @@
         <v>97671.45850214559</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>211285.7969410072</v>
+        <v>211285.8017876254</v>
       </c>
     </row>
     <row r="28">
@@ -4493,10 +4678,10 @@
         <v>989001946.7327092</v>
       </c>
       <c r="I28" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J28" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K28" t="n">
         <v>0</v>
@@ -4511,7 +4696,7 @@
         <v>97665.62476586687</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>211285.7969410072</v>
+        <v>211285.8017876254</v>
       </c>
     </row>
     <row r="29">
@@ -4542,10 +4727,10 @@
         <v>970100207.7670031</v>
       </c>
       <c r="I29" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J29" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K29" t="n">
         <v>0</v>
@@ -4560,7 +4745,7 @@
         <v>95799.04588667894</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>211413.0312696948</v>
+        <v>211413.0361217927</v>
       </c>
     </row>
     <row r="30">
@@ -4591,10 +4776,10 @@
         <v>970100207.7670031</v>
       </c>
       <c r="I30" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J30" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K30" t="n">
         <v>0</v>
@@ -4609,7 +4794,7 @@
         <v>95799.04588667894</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>211413.0312696948</v>
+        <v>211413.0361217927</v>
       </c>
     </row>
     <row r="31">
@@ -4640,10 +4825,10 @@
         <v>1003411510.006862</v>
       </c>
       <c r="I31" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J31" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K31" t="n">
         <v>0</v>
@@ -4655,10 +4840,10 @@
         <v>0.0367</v>
       </c>
       <c r="N31" s="3" t="n">
-        <v>99146.30231405739</v>
+        <v>99146.30233105208</v>
       </c>
       <c r="O31" s="3" t="n">
-        <v>215287.8949160884</v>
+        <v>215287.899935069</v>
       </c>
     </row>
     <row r="32">
@@ -4689,10 +4874,10 @@
         <v>983350180.9657269</v>
       </c>
       <c r="I32" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J32" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K32" t="n">
         <v>0</v>
@@ -4707,7 +4892,7 @@
         <v>97107.50328138829</v>
       </c>
       <c r="O32" s="3" t="n">
-        <v>215287.8949160884</v>
+        <v>215287.899935069</v>
       </c>
     </row>
     <row r="33">
@@ -4738,10 +4923,10 @@
         <v>1003284553.386072</v>
       </c>
       <c r="I33" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J33" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K33" t="n">
         <v>0</v>
@@ -4753,10 +4938,10 @@
         <v>0.0367</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>99131.61755004049</v>
+        <v>99131.61756640273</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>217601.2463467712</v>
+        <v>217601.2514653832</v>
       </c>
     </row>
     <row r="34">
@@ -4787,10 +4972,10 @@
         <v>1005279794.49182</v>
       </c>
       <c r="I34" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J34" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K34" t="n">
         <v>0</v>
@@ -4802,10 +4987,10 @@
         <v>0.0367</v>
       </c>
       <c r="N34" s="3" t="n">
-        <v>99362.40224336745</v>
+        <v>99362.40226966912</v>
       </c>
       <c r="O34" s="3" t="n">
-        <v>220151.9476342421</v>
+        <v>220151.9528627076</v>
       </c>
     </row>
     <row r="35">
@@ -4836,10 +5021,10 @@
         <v>985212276.3484071</v>
       </c>
       <c r="I35" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J35" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K35" t="n">
         <v>0</v>
@@ -4854,7 +5039,7 @@
         <v>97291.38836829222</v>
       </c>
       <c r="O35" s="3" t="n">
-        <v>220151.9476342421</v>
+        <v>220151.9528627076</v>
       </c>
     </row>
     <row r="36">
@@ -4885,10 +5070,10 @@
         <v>985212276.3484071</v>
       </c>
       <c r="I36" s="6" t="n">
-        <v>0.04</v>
+        <v>0.04000000189078801</v>
       </c>
       <c r="J36" s="6" t="n">
-        <v>0.04312</v>
+        <v>0.04312000189646037</v>
       </c>
       <c r="K36" t="n">
         <v>0</v>
@@ -4903,11 +5088,11 @@
         <v>97291.38836829222</v>
       </c>
       <c r="O36" s="3" t="n">
-        <v>220151.9476342421</v>
+        <v>220151.9528627076</v>
       </c>
     </row>
     <row r="38">
-      <c r="A38" s="8" t="inlineStr">
+      <c r="A38" s="7" t="inlineStr">
         <is>
           <t>Σ daily charges</t>
         </is>
@@ -4925,10 +5110,10 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="10" t="n">
-        <v>3322924.199551741</v>
+        <v>3322924.21170079</v>
       </c>
       <c r="O38" s="10" t="n">
-        <v>6577707.668676052</v>
+        <v>6577707.820120571</v>
       </c>
     </row>
   </sheetData>
@@ -5266,7 +5451,7 @@
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="8" t="inlineStr">
+      <c r="A5" s="7" t="inlineStr">
         <is>
           <t>E8 — Janus Henderson Anemoy AAA CLO (JAAA)</t>
         </is>

</xml_diff>

<commit_message>
chore(reports): regenerate under reconciled Cat A semantics
Restates Spark 2026-05 (S27 −$194,444.44 phantom yield → $0; supply-side
2,768,356.15 → 2,962,800.60) and Grove 2026-01/02 (E31/E32 re-bucketed to
capital); per-venue CoF allocations re-timed by the dated capital series.

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3270233.046142676</v>
+        <v>3270139.636212674</v>
       </c>
     </row>
     <row r="5">
@@ -508,7 +508,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3276508.572267083</v>
+        <v>3276415.162337082</v>
       </c>
     </row>
     <row r="8">
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>3270233.046142676</v>
+        <v>3270139.636212674</v>
       </c>
     </row>
     <row r="20">
@@ -622,7 +622,7 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>-52691.16555811382</v>
+        <v>-52784.57548811532</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-09T08:00:50+00:00</t>
+          <t>2026-07-10T11:17:30+00:00</t>
         </is>
       </c>
     </row>
@@ -854,13 +854,13 @@
         <v>0.3949353765426448</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>667436.8266593353</v>
+        <v>667441.0624591416</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2097307.010049039</v>
+        <v>2097311.245848845</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>265862.357248272</v>
+        <v>265858.1214484657</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>325000000</v>
@@ -992,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>804560.3212819771</v>
+        <v>804565.4273179597</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>804560.3212819771</v>
+        <v>804565.4273179597</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>240035.7851227842</v>
+        <v>240030.6790868015</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1057,13 +1057,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>782299.7953473206</v>
+        <v>782304.760109811</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>782299.7953473206</v>
+        <v>782304.760109811</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-547300.228786882</v>
+        <v>-547305.1935493723</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1191,13 +1191,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>315433.0136777532</v>
+        <v>315435.0155317787</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>315433.0136777532</v>
+        <v>315435.0155317787</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>300954.8863222468</v>
+        <v>300952.8844682213</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1256,13 +1256,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>230521.3992313645</v>
+        <v>230522.8622050261</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>230521.3992313645</v>
+        <v>230522.8622050261</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-124801.5267217337</v>
+        <v>-124802.9896953954</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1321,13 +1321,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>160722.5740597429</v>
+        <v>160723.5940643649</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>160722.5740597429</v>
+        <v>160723.5940643649</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>-91502.87984430196</v>
+        <v>-91503.89984892395</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1386,13 +1386,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>157716.5068388766</v>
+        <v>157717.5077658894</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>157716.5068388766</v>
+        <v>157717.5077658894</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>51419.74316112341</v>
+        <v>51418.74223411064</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1455,13 +1455,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78858.25341943829</v>
+        <v>78858.75388294469</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78858.25341943829</v>
+        <v>78858.75388294469</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-78858.25341943829</v>
+        <v>-78858.75388294469</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1524,13 +1524,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>78148.08204197524</v>
+        <v>78148.57799847263</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>78148.08204197524</v>
+        <v>78148.57799847263</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-76760.90570797524</v>
+        <v>-76761.40166447264</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1589,13 +1589,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>35689.80652831603</v>
+        <v>35690.03302896679</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>35689.80652831603</v>
+        <v>35690.03302896679</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>8322.66345968397</v>
+        <v>8322.436959033208</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1654,13 +1654,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10174.98964837061</v>
+        <v>10175.05422260065</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>10174.98964837061</v>
+        <v>10175.05422260065</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-134.3719947606131</v>
+        <v>-134.4365689906533</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1719,13 +1719,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1322.807713469469</v>
+        <v>1322.816108494186</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1322.807713469469</v>
+        <v>1322.816108494186</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>17.99092571625827</v>
+        <v>17.98253069154173</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1738,12 +1738,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>E15</t>
+          <t>E31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>AUSD raw (alt holder idle)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1757,40 +1757,40 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0</v>
+        <v>0.07814599999999999</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0</v>
+        <v>3688.95154</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0</v>
+        <v>3688.873394</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>1.5e-09</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>1.5e-09</v>
+        <v>0</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>6778.939209030984</v>
+        <v>3688.95154</v>
       </c>
       <c r="M16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>21.38301224242928</v>
+        <v>11.63624486315879</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>21.38301224242928</v>
+        <v>11.63624486315879</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-21.38301224092928</v>
+        <v>-11.63624486315879</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1831,31 +1831,31 @@
         <v>-3595.463464</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-3595.463464</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>-3595.463464</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>5849.73459</v>
+        <v>2254.271126</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>18.45199410938696</v>
+        <v>7.110760476426503</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>18.45199410938696</v>
+        <v>7.110760476426503</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-3613.915458109387</v>
+        <v>-7.110760476426503</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1868,12 +1868,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E31</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AUSD raw (alt holder idle)</t>
+          <t>Grove x Steakhouse USDC (Morpho 4626)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1883,44 +1883,44 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.07814599999999999</v>
+        <v>0</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>3688.95154</v>
+        <v>0</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0.07814599999999999</v>
+        <v>0</v>
       </c>
       <c r="M18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.000246498282868617</v>
+        <v>0</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.000246498282868617</v>
+        <v>0</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>3688.873147501717</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1933,12 +1933,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse USDC (Morpho 4626)</t>
+          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1998,12 +1998,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2063,12 +2063,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E37</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maple syrupUSDC (ERC-4626)</t>
+          <t>Curve AUSD/USDC stableswap LP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
@@ -2128,12 +2128,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Curve AUSD/USDC stableswap LP</t>
+          <t>RLUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -2193,12 +2193,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">

</xml_diff>

<commit_message>
fix(cat-a): reconcile idle par-stable revenue via explicit external_yield_source (supersedes #148, #151) (#153)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -492,7 +492,7 @@
         </is>
       </c>
       <c r="B4" s="3" t="n">
-        <v>3270233.046142676</v>
+        <v>3270139.636212674</v>
       </c>
     </row>
     <row r="5">
@@ -508,7 +508,7 @@
     <row r="6">
       <c r="A6" t="inlineStr"/>
       <c r="B6" s="4" t="n">
-        <v>3276508.572267083</v>
+        <v>3276415.162337082</v>
       </c>
     </row>
     <row r="8">
@@ -606,7 +606,7 @@
         </is>
       </c>
       <c r="B19" s="3" t="n">
-        <v>3270233.046142676</v>
+        <v>3270139.636212674</v>
       </c>
     </row>
     <row r="20">
@@ -622,7 +622,7 @@
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>-52691.16555811382</v>
+        <v>-52784.57548811532</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-07T14:51:35+00:00</t>
+          <t>2026-07-10T11:17:30+00:00</t>
         </is>
       </c>
     </row>
@@ -854,13 +854,13 @@
         <v>0.3949353765426448</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>667436.8266593353</v>
+        <v>667441.0624591416</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2097307.010049039</v>
+        <v>2097311.245848845</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>265862.357248272</v>
+        <v>265858.1214484657</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>325000000</v>
@@ -992,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>804560.3212819771</v>
+        <v>804565.4273179597</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>804560.3212819771</v>
+        <v>804565.4273179597</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>240035.7851227842</v>
+        <v>240030.6790868015</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1057,13 +1057,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>782299.7953473206</v>
+        <v>782304.760109811</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>782299.7953473206</v>
+        <v>782304.760109811</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-547300.228786882</v>
+        <v>-547305.1935493723</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1191,13 +1191,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>315433.0136777532</v>
+        <v>315435.0155317787</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>315433.0136777532</v>
+        <v>315435.0155317787</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>300954.8863222468</v>
+        <v>300952.8844682213</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1256,13 +1256,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>230521.3992313645</v>
+        <v>230522.8622050261</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>230521.3992313645</v>
+        <v>230522.8622050261</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-124801.5267217337</v>
+        <v>-124802.9896953954</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1321,13 +1321,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>160722.5740597429</v>
+        <v>160723.5940643649</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>160722.5740597429</v>
+        <v>160723.5940643649</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>-91502.87984430196</v>
+        <v>-91503.89984892395</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1386,13 +1386,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>157716.5068388766</v>
+        <v>157717.5077658894</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>157716.5068388766</v>
+        <v>157717.5077658894</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>51419.74316112341</v>
+        <v>51418.74223411064</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1455,13 +1455,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78858.25341943829</v>
+        <v>78858.75388294469</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78858.25341943829</v>
+        <v>78858.75388294469</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-78858.25341943829</v>
+        <v>-78858.75388294469</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1524,13 +1524,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>78148.08204197524</v>
+        <v>78148.57799847263</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>78148.08204197524</v>
+        <v>78148.57799847263</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-76760.90570797524</v>
+        <v>-76761.40166447264</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1589,13 +1589,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>35689.80652831603</v>
+        <v>35690.03302896679</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>35689.80652831603</v>
+        <v>35690.03302896679</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>8322.66345968397</v>
+        <v>8322.436959033208</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1654,13 +1654,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10174.98964837061</v>
+        <v>10175.05422260065</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>10174.98964837061</v>
+        <v>10175.05422260065</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-134.3719947606131</v>
+        <v>-134.4365689906533</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1719,13 +1719,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1322.807713469469</v>
+        <v>1322.816108494186</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1322.807713469469</v>
+        <v>1322.816108494186</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>17.99092571625827</v>
+        <v>17.98253069154173</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1738,12 +1738,12 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>E15</t>
+          <t>E31</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>USDC raw (ALM idle)</t>
+          <t>AUSD raw (alt holder idle)</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -1757,40 +1757,40 @@
         </is>
       </c>
       <c r="E16" s="5" t="n">
-        <v>0</v>
+        <v>0.07814599999999999</v>
       </c>
       <c r="F16" s="5" t="n">
-        <v>0</v>
+        <v>3688.95154</v>
       </c>
       <c r="G16" s="5" t="n">
-        <v>0</v>
+        <v>3688.873394</v>
       </c>
       <c r="H16" s="5" t="n">
-        <v>1.5e-09</v>
+        <v>0</v>
       </c>
       <c r="I16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J16" s="5" t="n">
-        <v>1.5e-09</v>
+        <v>0</v>
       </c>
       <c r="K16" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L16" s="5" t="n">
-        <v>6778.939209030984</v>
+        <v>3688.95154</v>
       </c>
       <c r="M16" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>21.38301224242928</v>
+        <v>11.63624486315879</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>21.38301224242928</v>
+        <v>11.63624486315879</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-21.38301224092928</v>
+        <v>-11.63624486315879</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1831,31 +1831,31 @@
         <v>-3595.463464</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>-3595.463464</v>
+        <v>0</v>
       </c>
       <c r="I17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J17" s="5" t="n">
-        <v>-3595.463464</v>
+        <v>0</v>
       </c>
       <c r="K17" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L17" s="5" t="n">
-        <v>5849.73459</v>
+        <v>2254.271126</v>
       </c>
       <c r="M17" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>18.45199410938696</v>
+        <v>7.110760476426503</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>18.45199410938696</v>
+        <v>7.110760476426503</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-3613.915458109387</v>
+        <v>-7.110760476426503</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -1868,12 +1868,12 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>E31</t>
+          <t>E4</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>AUSD raw (alt holder idle)</t>
+          <t>Grove x Steakhouse USDC (Morpho 4626)</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
@@ -1883,44 +1883,44 @@
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>B</t>
         </is>
       </c>
       <c r="E18" s="5" t="n">
-        <v>0.07814599999999999</v>
+        <v>0</v>
       </c>
       <c r="F18" s="5" t="n">
-        <v>3688.95154</v>
+        <v>0</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="H18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="I18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="J18" s="5" t="n">
-        <v>3688.873394</v>
+        <v>0</v>
       </c>
       <c r="K18" s="5" t="n">
         <v>0</v>
       </c>
       <c r="L18" s="5" t="n">
-        <v>0.07814599999999999</v>
+        <v>0</v>
       </c>
       <c r="M18" s="6" t="n">
         <v>1</v>
       </c>
       <c r="N18" s="5" t="n">
-        <v>0.000246498282868617</v>
+        <v>0</v>
       </c>
       <c r="O18" s="5" t="n">
-        <v>0.000246498282868617</v>
+        <v>0</v>
       </c>
       <c r="P18" s="5" t="n">
-        <v>3688.873147501717</v>
+        <v>0</v>
       </c>
       <c r="Q18" s="5" t="n">
         <v>0</v>
@@ -1933,12 +1933,12 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>E4</t>
+          <t>E6</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse USDC (Morpho 4626)</t>
+          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -1998,12 +1998,12 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>E6</t>
+          <t>E37</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Grove x Steakhouse AUSD (Morpho 4626)</t>
+          <t>Maple syrupUSDC (ERC-4626)</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -2063,12 +2063,12 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>E37</t>
+          <t>E11</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Maple syrupUSDC (ERC-4626)</t>
+          <t>Curve AUSD/USDC stableswap LP</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
@@ -2078,7 +2078,7 @@
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>B</t>
+          <t>F</t>
         </is>
       </c>
       <c r="E21" s="5" t="n">
@@ -2128,12 +2128,12 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>E11</t>
+          <t>E13</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Curve AUSD/USDC stableswap LP</t>
+          <t>RLUSD raw (ALM idle)</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
@@ -2143,7 +2143,7 @@
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>F</t>
+          <t>A</t>
         </is>
       </c>
       <c r="E22" s="5" t="n">
@@ -2193,12 +2193,12 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>E13</t>
+          <t>E15</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>RLUSD raw (ALM idle)</t>
+          <t>USDC raw (ALM idle)</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">

</xml_diff>

<commit_message>
feat(spark): EFFR → 3M T-Bill + HyperSync debt; fix fabricated T-Bill data (Spark + Grove) (#159)
Co-authored-by: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -1,19 +1,19 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Venues" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Debt" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Off-protocol holdings" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="SDE daily" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Summary" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Venues" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Sky Revenue" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Sky Direct" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Debt" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Off-protocol holdings" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="SDE daily" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -530,7 +530,7 @@
         </is>
       </c>
       <c r="B9" s="3" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
     </row>
     <row r="10">
@@ -546,7 +546,7 @@
     <row r="11">
       <c r="A11" t="inlineStr"/>
       <c r="B11" s="4" t="n">
-        <v>6277336.089037795</v>
+        <v>6272709.564932599</v>
       </c>
     </row>
     <row r="13">
@@ -568,7 +568,7 @@
         </is>
       </c>
       <c r="B14" s="3" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
     </row>
     <row r="15">
@@ -578,13 +578,13 @@
         </is>
       </c>
       <c r="B15" s="3" t="n">
-        <v>-3254783.608419782</v>
+        <v>-3254914.174321245</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
       <c r="B16" s="4" t="n">
-        <v>6577707.820120571</v>
+        <v>6573211.86191684</v>
       </c>
     </row>
     <row r="18">
@@ -616,13 +616,13 @@
         </is>
       </c>
       <c r="B20" s="3" t="n">
-        <v>-3322924.21170079</v>
+        <v>-3318297.687595594</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr"/>
       <c r="B21" s="4" t="n">
-        <v>-52784.57548811532</v>
+        <v>-48158.05138291954</v>
       </c>
     </row>
     <row r="23">
@@ -657,7 +657,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>2026-07-10T11:17:30+00:00</t>
+          <t>2026-07-31T00:07:04+00:00</t>
         </is>
       </c>
     </row>
@@ -854,13 +854,13 @@
         <v>0.3949353765426448</v>
       </c>
       <c r="N2" s="5" t="n">
-        <v>667441.0624591416</v>
+        <v>666511.7809084547</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>2097311.245848845</v>
+        <v>2096381.964298158</v>
       </c>
       <c r="P2" s="5" t="n">
-        <v>265858.1214484657</v>
+        <v>266787.4029991527</v>
       </c>
       <c r="Q2" s="5" t="n">
         <v>325000000</v>
@@ -992,13 +992,13 @@
         <v>1</v>
       </c>
       <c r="N4" s="5" t="n">
-        <v>804565.4273179597</v>
+        <v>803445.2268238929</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>804565.4273179597</v>
+        <v>803445.2268238929</v>
       </c>
       <c r="P4" s="5" t="n">
-        <v>240030.6790868015</v>
+        <v>241150.8795808683</v>
       </c>
       <c r="Q4" s="5" t="n">
         <v>0</v>
@@ -1057,13 +1057,13 @@
         <v>1</v>
       </c>
       <c r="N5" s="5" t="n">
-        <v>782304.760109811</v>
+        <v>781215.5532547425</v>
       </c>
       <c r="O5" s="5" t="n">
-        <v>782304.760109811</v>
+        <v>781215.5532547425</v>
       </c>
       <c r="P5" s="5" t="n">
-        <v>-547305.1935493723</v>
+        <v>-546215.9866943038</v>
       </c>
       <c r="Q5" s="5" t="n">
         <v>0</v>
@@ -1191,13 +1191,13 @@
         <v>1</v>
       </c>
       <c r="N7" s="5" t="n">
-        <v>315435.0155317787</v>
+        <v>314995.8337719776</v>
       </c>
       <c r="O7" s="5" t="n">
-        <v>315435.0155317787</v>
+        <v>314995.8337719776</v>
       </c>
       <c r="P7" s="5" t="n">
-        <v>300952.8844682213</v>
+        <v>301392.0662280224</v>
       </c>
       <c r="Q7" s="5" t="n">
         <v>0</v>
@@ -1256,13 +1256,13 @@
         <v>1</v>
       </c>
       <c r="N8" s="5" t="n">
-        <v>230522.8622050261</v>
+        <v>230201.9040636894</v>
       </c>
       <c r="O8" s="5" t="n">
-        <v>230522.8622050261</v>
+        <v>230201.9040636894</v>
       </c>
       <c r="P8" s="5" t="n">
-        <v>-124802.9896953954</v>
+        <v>-124482.0315540587</v>
       </c>
       <c r="Q8" s="5" t="n">
         <v>0</v>
@@ -1321,13 +1321,13 @@
         <v>1</v>
       </c>
       <c r="N9" s="5" t="n">
-        <v>160723.5940643649</v>
+        <v>160499.8177953805</v>
       </c>
       <c r="O9" s="5" t="n">
-        <v>160723.5940643649</v>
+        <v>160499.8177953805</v>
       </c>
       <c r="P9" s="5" t="n">
-        <v>-91503.89984892395</v>
+        <v>-91280.12357993951</v>
       </c>
       <c r="Q9" s="5" t="n">
         <v>0</v>
@@ -1386,13 +1386,13 @@
         <v>1</v>
       </c>
       <c r="N10" s="5" t="n">
-        <v>157717.5077658894</v>
+        <v>157497.9168859888</v>
       </c>
       <c r="O10" s="5" t="n">
-        <v>157717.5077658894</v>
+        <v>157497.9168859888</v>
       </c>
       <c r="P10" s="5" t="n">
-        <v>51418.74223411064</v>
+        <v>51638.33311401121</v>
       </c>
       <c r="Q10" s="5" t="n">
         <v>0</v>
@@ -1455,13 +1455,13 @@
         <v>1</v>
       </c>
       <c r="N11" s="5" t="n">
-        <v>78858.75388294469</v>
+        <v>78748.95844299439</v>
       </c>
       <c r="O11" s="5" t="n">
-        <v>78858.75388294469</v>
+        <v>78748.95844299439</v>
       </c>
       <c r="P11" s="5" t="n">
-        <v>-78858.75388294469</v>
+        <v>-78748.95844299439</v>
       </c>
       <c r="Q11" s="5" t="n">
         <v>0</v>
@@ -1524,13 +1524,13 @@
         <v>1</v>
       </c>
       <c r="N12" s="5" t="n">
-        <v>78148.57799847263</v>
+        <v>78039.77133998081</v>
       </c>
       <c r="O12" s="5" t="n">
-        <v>78148.57799847263</v>
+        <v>78039.77133998081</v>
       </c>
       <c r="P12" s="5" t="n">
-        <v>-76761.40166447264</v>
+        <v>-76652.59500598082</v>
       </c>
       <c r="Q12" s="5" t="n">
         <v>0</v>
@@ -1589,13 +1589,13 @@
         <v>1</v>
       </c>
       <c r="N13" s="5" t="n">
-        <v>35690.03302896679</v>
+        <v>35640.34161634224</v>
       </c>
       <c r="O13" s="5" t="n">
-        <v>35690.03302896679</v>
+        <v>35640.34161634224</v>
       </c>
       <c r="P13" s="5" t="n">
-        <v>8322.436959033208</v>
+        <v>8372.128371657764</v>
       </c>
       <c r="Q13" s="5" t="n">
         <v>0</v>
@@ -1654,13 +1654,13 @@
         <v>1</v>
       </c>
       <c r="N14" s="5" t="n">
-        <v>10175.05422260065</v>
+        <v>10160.88744339252</v>
       </c>
       <c r="O14" s="5" t="n">
-        <v>10175.05422260065</v>
+        <v>10160.88744339252</v>
       </c>
       <c r="P14" s="5" t="n">
-        <v>-134.4365689906533</v>
+        <v>-120.2697897825169</v>
       </c>
       <c r="Q14" s="5" t="n">
         <v>0</v>
@@ -1719,13 +1719,13 @@
         <v>1</v>
       </c>
       <c r="N15" s="5" t="n">
-        <v>1322.816108494186</v>
+        <v>1320.974344968211</v>
       </c>
       <c r="O15" s="5" t="n">
-        <v>1322.816108494186</v>
+        <v>1320.974344968211</v>
       </c>
       <c r="P15" s="5" t="n">
-        <v>17.98253069154173</v>
+        <v>19.8242942175167</v>
       </c>
       <c r="Q15" s="5" t="n">
         <v>0</v>
@@ -1784,13 +1784,13 @@
         <v>1</v>
       </c>
       <c r="N16" s="5" t="n">
-        <v>11.63624486315879</v>
+        <v>11.62004366086721</v>
       </c>
       <c r="O16" s="5" t="n">
-        <v>11.63624486315879</v>
+        <v>11.62004366086721</v>
       </c>
       <c r="P16" s="5" t="n">
-        <v>-11.63624486315879</v>
+        <v>-11.62004366086721</v>
       </c>
       <c r="Q16" s="5" t="n">
         <v>0</v>
@@ -1849,13 +1849,13 @@
         <v>1</v>
       </c>
       <c r="N17" s="5" t="n">
-        <v>7.110760476426503</v>
+        <v>7.100860128824647</v>
       </c>
       <c r="O17" s="5" t="n">
-        <v>7.110760476426503</v>
+        <v>7.100860128824647</v>
       </c>
       <c r="P17" s="5" t="n">
-        <v>-7.110760476426503</v>
+        <v>-7.100860128824647</v>
       </c>
       <c r="Q17" s="5" t="n">
         <v>0</v>
@@ -2931,7 +2931,7 @@
         </is>
       </c>
       <c r="B9" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.03664516129032258</v>
       </c>
     </row>
     <row r="10">
@@ -2941,7 +2941,7 @@
         </is>
       </c>
       <c r="B10" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.03664516129032258</v>
       </c>
     </row>
     <row r="11">
@@ -2951,7 +2951,7 @@
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>0.03717115181169214</v>
+        <v>0.03711850878908277</v>
       </c>
     </row>
     <row r="12">
@@ -2961,7 +2961,7 @@
         </is>
       </c>
       <c r="B12" s="9" t="n">
-        <v>-59.48850084768234</v>
+        <v>-60.01493107377607</v>
       </c>
     </row>
     <row r="13">
@@ -2971,7 +2971,7 @@
         </is>
       </c>
       <c r="B13" s="10" t="n">
-        <v>520885.9412035887</v>
+        <v>525512.4653087845</v>
       </c>
     </row>
     <row r="15">
@@ -2991,7 +2991,7 @@
         </is>
       </c>
       <c r="B16" s="3" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
     </row>
     <row r="17">
@@ -3001,7 +3001,7 @@
         </is>
       </c>
       <c r="B17" s="10" t="n">
-        <v>520885.9412035887</v>
+        <v>525512.4653087845</v>
       </c>
     </row>
     <row r="19">
@@ -3031,7 +3031,7 @@
         <v>993313796.6169302</v>
       </c>
       <c r="C20" s="3" t="n">
-        <v>3040834.245599687</v>
+        <v>3036207.721494491</v>
       </c>
     </row>
     <row r="21">
@@ -3066,7 +3066,7 @@
         </is>
       </c>
       <c r="B24" s="3" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
     </row>
     <row r="25">
@@ -3086,7 +3086,7 @@
         </is>
       </c>
       <c r="B26" s="3" t="n">
-        <v>6277336.089037795</v>
+        <v>6272709.564932599</v>
       </c>
     </row>
     <row r="28">
@@ -3103,7 +3103,7 @@
         </is>
       </c>
       <c r="B30" s="3" t="n">
-        <v>6577707.820120571</v>
+        <v>6573211.86191684</v>
       </c>
     </row>
     <row r="31">
@@ -3113,7 +3113,7 @@
         </is>
       </c>
       <c r="B31" s="3" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
     </row>
     <row r="32">
@@ -3123,7 +3123,7 @@
         </is>
       </c>
       <c r="B32" s="3" t="n">
-        <v>-3254783.608419782</v>
+        <v>-3254914.174321245</v>
       </c>
     </row>
     <row r="33" ht="60" customHeight="1">
@@ -3658,16 +3658,16 @@
         <v>0</v>
       </c>
       <c r="L7" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="M7" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="N7" s="3" t="n">
-        <v>124541.7904362082</v>
+        <v>124013.1398739934</v>
       </c>
       <c r="O7" s="3" t="n">
-        <v>212780.043244714</v>
+        <v>212251.3926824992</v>
       </c>
     </row>
     <row r="8">
@@ -3707,16 +3707,16 @@
         <v>0</v>
       </c>
       <c r="L8" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="M8" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="N8" s="3" t="n">
-        <v>124541.7904362082</v>
+        <v>124013.1398739934</v>
       </c>
       <c r="O8" s="3" t="n">
-        <v>212780.043244714</v>
+        <v>212251.3926824992</v>
       </c>
     </row>
     <row r="9">
@@ -3756,16 +3756,16 @@
         <v>0</v>
       </c>
       <c r="L9" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="M9" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0365</v>
       </c>
       <c r="N9" s="3" t="n">
-        <v>124537.2371181835</v>
+        <v>124008.5865559687</v>
       </c>
       <c r="O9" s="3" t="n">
-        <v>212780.043244714</v>
+        <v>212251.3926824992</v>
       </c>
     </row>
     <row r="10">
@@ -3805,16 +3805,16 @@
         <v>0</v>
       </c>
       <c r="L10" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0364</v>
       </c>
       <c r="M10" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0364</v>
       </c>
       <c r="N10" s="3" t="n">
-        <v>125679.7338753068</v>
+        <v>124886.719882834</v>
       </c>
       <c r="O10" s="3" t="n">
-        <v>213936.7190098711</v>
+        <v>213143.7050173984</v>
       </c>
     </row>
     <row r="11">
@@ -3854,16 +3854,16 @@
         <v>0</v>
       </c>
       <c r="L11" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0363</v>
       </c>
       <c r="M11" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0363</v>
       </c>
       <c r="N11" s="3" t="n">
-        <v>127583.5807271658</v>
+        <v>126526.1778654509</v>
       </c>
       <c r="O11" s="3" t="n">
-        <v>215845.2340223803</v>
+        <v>214787.8311606654</v>
       </c>
     </row>
     <row r="12">
@@ -3903,16 +3903,16 @@
         <v>0</v>
       </c>
       <c r="L12" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="M12" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="N12" s="3" t="n">
-        <v>122286.8068660209</v>
+        <v>120964.9896907505</v>
       </c>
       <c r="O12" s="3" t="n">
-        <v>215180.0281722427</v>
+        <v>213858.2109969723</v>
       </c>
     </row>
     <row r="13">
@@ -3952,16 +3952,16 @@
         <v>0</v>
       </c>
       <c r="L13" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="M13" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="N13" s="3" t="n">
-        <v>124595.6621390942</v>
+        <v>123273.8449638237</v>
       </c>
       <c r="O13" s="3" t="n">
-        <v>217493.3797025569</v>
+        <v>216171.5625272865</v>
       </c>
     </row>
     <row r="14">
@@ -4001,16 +4001,16 @@
         <v>0</v>
       </c>
       <c r="L14" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="M14" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="N14" s="3" t="n">
-        <v>110704.6990285211</v>
+        <v>109382.8818532506</v>
       </c>
       <c r="O14" s="3" t="n">
-        <v>205920.5980230453</v>
+        <v>204598.7808477748</v>
       </c>
     </row>
     <row r="15">
@@ -4050,16 +4050,16 @@
         <v>0</v>
       </c>
       <c r="L15" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="M15" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="N15" s="3" t="n">
-        <v>110704.6990285211</v>
+        <v>109382.8818532506</v>
       </c>
       <c r="O15" s="3" t="n">
-        <v>205920.5980230453</v>
+        <v>204598.7808477748</v>
       </c>
     </row>
     <row r="16">
@@ -4099,16 +4099,16 @@
         <v>0</v>
       </c>
       <c r="L16" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="M16" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0362</v>
       </c>
       <c r="N16" s="3" t="n">
-        <v>110704.6990285211</v>
+        <v>109382.8818532506</v>
       </c>
       <c r="O16" s="3" t="n">
-        <v>205920.5980230453</v>
+        <v>204598.7808477748</v>
       </c>
     </row>
     <row r="17">
@@ -4295,16 +4295,16 @@
         <v>0</v>
       </c>
       <c r="L20" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0368</v>
       </c>
       <c r="M20" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0368</v>
       </c>
       <c r="N20" s="3" t="n">
-        <v>100871.8172433724</v>
+        <v>101136.1043853213</v>
       </c>
       <c r="O20" s="3" t="n">
-        <v>209998.027425971</v>
+        <v>210262.31456792</v>
       </c>
     </row>
     <row r="21">
@@ -4540,16 +4540,16 @@
         <v>0</v>
       </c>
       <c r="L25" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="M25" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="N25" s="3" t="n">
-        <v>95806.17217862917</v>
+        <v>96575.31044899891</v>
       </c>
       <c r="O25" s="3" t="n">
-        <v>206774.7663035127</v>
+        <v>207567.5514754674</v>
       </c>
     </row>
     <row r="26">
@@ -4589,16 +4589,16 @@
         <v>0</v>
       </c>
       <c r="L26" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="M26" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="N26" s="3" t="n">
-        <v>93865.19116313005</v>
+        <v>94618.74710986516</v>
       </c>
       <c r="O26" s="3" t="n">
-        <v>206821.033334119</v>
+        <v>207613.8185060737</v>
       </c>
     </row>
     <row r="27">
@@ -4638,16 +4638,16 @@
         <v>0</v>
       </c>
       <c r="L27" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0371</v>
       </c>
       <c r="M27" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0371</v>
       </c>
       <c r="N27" s="3" t="n">
-        <v>97671.45850214559</v>
+        <v>98716.89211467199</v>
       </c>
       <c r="O27" s="3" t="n">
-        <v>211285.8017876254</v>
+        <v>212342.7978574069</v>
       </c>
     </row>
     <row r="28">
@@ -4687,16 +4687,16 @@
         <v>0</v>
       </c>
       <c r="L28" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="M28" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="N28" s="3" t="n">
-        <v>97665.62476586687</v>
+        <v>98449.6908442709</v>
       </c>
       <c r="O28" s="3" t="n">
-        <v>211285.8017876254</v>
+        <v>212078.5869595801</v>
       </c>
     </row>
     <row r="29">
@@ -4736,16 +4736,16 @@
         <v>0</v>
       </c>
       <c r="L29" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="M29" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="N29" s="3" t="n">
-        <v>95799.04588667894</v>
+        <v>96568.12694670679</v>
       </c>
       <c r="O29" s="3" t="n">
-        <v>211413.0361217927</v>
+        <v>212205.8212937474</v>
       </c>
     </row>
     <row r="30">
@@ -4785,16 +4785,16 @@
         <v>0</v>
       </c>
       <c r="L30" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="M30" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.037</v>
       </c>
       <c r="N30" s="3" t="n">
-        <v>95799.04588667894</v>
+        <v>96568.12694670679</v>
       </c>
       <c r="O30" s="3" t="n">
-        <v>211413.0361217927</v>
+        <v>212205.8212937474</v>
       </c>
     </row>
     <row r="31">
@@ -4932,16 +4932,16 @@
         <v>0</v>
       </c>
       <c r="L33" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0368</v>
       </c>
       <c r="M33" s="6" t="n">
-        <v>0.0367</v>
+        <v>0.0368</v>
       </c>
       <c r="N33" s="3" t="n">
-        <v>99131.61756640273</v>
+        <v>99395.90470835165</v>
       </c>
       <c r="O33" s="3" t="n">
-        <v>217601.2514653832</v>
+        <v>217865.5386073321</v>
       </c>
     </row>
     <row r="34">
@@ -5110,10 +5110,10 @@
       <c r="L38" t="inlineStr"/>
       <c r="M38" t="inlineStr"/>
       <c r="N38" s="10" t="n">
-        <v>3322924.21170079</v>
+        <v>3318297.687595594</v>
       </c>
       <c r="O38" s="10" t="n">
-        <v>6577707.820120571</v>
+        <v>6573211.86191684</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(msc11): July 2026 settlement cycle — 2026-07-23 rate regime, Osero + Grove Diamond PAU, spUSDG/Robinhood, DR, accrual sky_total (#164)
Co-authored-by: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
+++ b/settlements/grove/2026-01/grove_settlement_january_2026.xlsx
@@ -2917,7 +2917,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Base rate (BR = SSR + 30bps), period avg</t>
+          <t>Base rate (BR = SSR (+) spread; 30bps, 20bps from 2026-07-23), period avg</t>
         </is>
       </c>
       <c r="B8" s="6" t="n">
@@ -3197,7 +3197,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>tbill_3m</t>
+          <t>tbill_3m→sofr@2026-07-23</t>
         </is>
       </c>
     </row>
@@ -3228,7 +3228,7 @@
     <row r="44">
       <c r="A44" s="11" t="inlineStr">
         <is>
-          <t>Base rate composition: base_apy = (1 + SSR)(1 + 30bps) − 1 (multiplicative)</t>
+          <t>Base rate composition: base_apy = (1 + SSR)(1 + spread) − 1 (multiplicative; spread 30bps, 20bps from 2026-07-23)</t>
         </is>
       </c>
     </row>
@@ -3492,7 +3492,7 @@
     <row r="3" ht="45" customHeight="1">
       <c r="A3" s="12" t="inlineStr">
         <is>
-          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40), then scaled by Vat.ilks[ilk].rate_d / 1e27 read at each day's EoD block — actual outstanding USDS per day, not raw normalised Art. utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+0.003)−1 (multiplicative). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
+          <t>cum_debt = Σ on-chain Vat dart from frob (0x76088703) + grab (0x7bab3f40), then scaled by Vat.ilks[ilk].rate_d / 1e27 read at each day's EoD block — actual outstanding USDS per day, not raw normalised Art. utilized = cum_debt − Σ deductions. base_apy = (1+SSR)(1+spread)−1 (multiplicative; spread 30bps, 20bps from 2026-07-23). sub_apy applies on the first cap_usd of utilized when the subsidy is active; excess pays base_apy.</t>
         </is>
       </c>
     </row>

</xml_diff>